<commit_message>
Save current changes before cleaning history
</commit_message>
<xml_diff>
--- a/build/temp/pages/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
+++ b/build/temp/pages/StructureDefinition-cibmtr-additional-peri-transplant-medication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.9</t>
+    <t>0.1.11</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-09-19T15:08:00-05:00</t>
+    <t>2026-06-10T07:35:08-05:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -442,7 +442,7 @@
     <t>Medication.meta.profile</t>
   </si>
   <si>
-    <t xml:space="preserve">canonical(StructureDefinition)
+    <t xml:space="preserve">canonical(StructureDefinition|4.0.1)
 </t>
   </si>
   <si>
@@ -480,7 +480,7 @@
     <t>Security Labels from the Healthcare Privacy and Security Classification System.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/security-labels</t>
+    <t>http://hl7.org/fhir/ValueSet/security-labels|4.0.1</t>
   </si>
   <si>
     <t xml:space="preserve">pattern:system}
@@ -670,7 +670,7 @@
     <t>Codes that represent various types of tags, commonly workflow-related; e.g. "Needs review by Dr. Jones".</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/common-tags</t>
+    <t>http://hl7.org/fhir/ValueSet/common-tags|4.0.1</t>
   </si>
   <si>
     <t>Meta.tag</t>
@@ -1482,7 +1482,7 @@
     <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="28.53125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="30.03515625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -2769,7 +2769,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" hidden="true">
+    <row r="12">
       <c r="A12" t="s" s="2">
         <v>151</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" hidden="true">
+    <row r="28">
       <c r="A28" t="s" s="2">
         <v>255</v>
       </c>
@@ -7095,12 +7095,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AN49">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>